<commit_message>
Correction of range control
</commit_message>
<xml_diff>
--- a/data/result/validation_errors.xlsx
+++ b/data/result/validation_errors.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -520,7 +520,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -908,7 +908,7 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -918,21 +918,21 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>74904</v>
+        <v>60758</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>branch</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>1/91/2024</t>
+          <t>5656565</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>INVALID_DATE</t>
+          <t>BUSINESS_RULE_VIOLATION</t>
         </is>
       </c>
       <c r="E19" t="n">
@@ -940,87 +940,303 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Value '1/91/2024' is not a valid date. Please use YYYY-MM-DD or DD/MM/YYYY.</t>
+          <t>Value 5656565 must be between 1 and 2999 for branch</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>74955</v>
+        <v>74904</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>branch</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ff</t>
+          <t>1/91/2024</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>TYPE_MISMATCH</t>
+          <t>INVALID_DATE</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Expected float but got: 'ff'</t>
+          <t>Value '1/91/2024' is not a valid date. Please use YYYY-MM-DD or DD/MM/YYYY.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>75004</v>
+        <v>74905</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>amount</t>
+          <t>branch</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>df</t>
+          <t>545454</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>TYPE_MISMATCH</t>
+          <t>BUSINESS_RULE_VIOLATION</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Expected float but got: 'df'</t>
+          <t>Value 545454 must be between 1 and 2999 for branch</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
+        <v>74955</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>branch</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>ff</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>TYPE_MISMATCH</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Expected float but got: 'ff'</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>74966</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>branch</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>5251502525</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>BUSINESS_RULE_VIOLATION</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>3</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Value 5251502525 must be between 1 and 2999 for branch</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>75004</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>df</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>TYPE_MISMATCH</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>2</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Expected float but got: 'df'</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
         <v>75005</v>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>amount</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr">
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr">
         <is>
           <t>MISSING_REQUIRED</t>
         </is>
       </c>
-      <c r="E22" t="n">
+      <c r="E25" t="n">
         <v>2</v>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>Mandatory field is empty</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>435</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>invoice_number</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>inv-432</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>COMPOSITE_DUPLICATE</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Original row flagged: Conflict with row 75006</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>75006</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>invoice_number</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>INV-432</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>COMPOSITE_DUPLICATE</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Duplicate of row 435</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>75007</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>MISSING_REQUIRED</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>2</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Mandatory field is empty</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>75008</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>MISSING_REQUIRED</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>2</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Mandatory field is empty</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>75008</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>سی</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>TYPE_MISMATCH</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>2</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Expected float but got: 'سی'</t>
         </is>
       </c>
     </row>

</xml_diff>